<commit_message>
Fix CORS issue for Render deployment
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -872,268 +872,268 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>33.66950225830078</v>
+        <v>32.37878799438477</v>
       </c>
       <c r="B2" t="n">
-        <v>0.2243958860635757</v>
+        <v>0.1399308443069458</v>
       </c>
       <c r="C2" t="n">
-        <v>32.72253799438477</v>
+        <v>31.48935699462891</v>
       </c>
       <c r="D2" t="n">
-        <v>37.15348052978516</v>
+        <v>32.65531539916992</v>
       </c>
       <c r="E2" t="n">
-        <v>38.20817565917969</v>
+        <v>33.95757675170898</v>
       </c>
       <c r="F2" t="n">
-        <v>5.485637664794922</v>
+        <v>2.468219757080078</v>
       </c>
       <c r="G2" t="n">
-        <v>164.6822204589844</v>
+        <v>123.0326080322266</v>
       </c>
       <c r="H2" t="n">
-        <v>85.63771820068359</v>
+        <v>97.15403747558594</v>
       </c>
       <c r="I2" t="n">
-        <v>59.71787643432617</v>
+        <v>26.1563606262207</v>
       </c>
       <c r="J2" t="n">
-        <v>39.5915641784668</v>
+        <v>14.35910224914551</v>
       </c>
       <c r="K2" t="n">
-        <v>1.308539271354675</v>
+        <v>0.7915711402893066</v>
       </c>
       <c r="L2" t="n">
-        <v>0.8515964150428772</v>
+        <v>0.7487615942955017</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2139041125774384</v>
+        <v>0.2599876224994659</v>
       </c>
       <c r="N2" t="n">
-        <v>1.005673408508301</v>
+        <v>0.6808357238769531</v>
       </c>
       <c r="O2" t="n">
-        <v>2.310833215713501</v>
+        <v>1.196025133132935</v>
       </c>
       <c r="P2" t="n">
-        <v>2.09692907333374</v>
+        <v>0.936037540435791</v>
       </c>
       <c r="Q2" t="n">
-        <v>14.39002513885498</v>
+        <v>16.84541511535645</v>
       </c>
       <c r="R2" t="n">
-        <v>5.022202491760254</v>
+        <v>12.32826614379883</v>
       </c>
       <c r="S2" t="n">
-        <v>11.6517276763916</v>
+        <v>10.85582828521729</v>
       </c>
       <c r="T2" t="n">
-        <v>4.771716594696045</v>
+        <v>8.22602653503418</v>
       </c>
       <c r="U2" t="n">
-        <v>0.924603283405304</v>
+        <v>0.5492869019508362</v>
       </c>
       <c r="V2" t="n">
-        <v>0.9340814352035522</v>
+        <v>1.099833011627197</v>
       </c>
       <c r="W2" t="n">
-        <v>24.56069946289062</v>
+        <v>21.01264381408691</v>
       </c>
       <c r="X2" t="n">
-        <v>0.8374003171920776</v>
+        <v>1.111422657966614</v>
       </c>
       <c r="Y2" t="n">
-        <v>14.64946556091309</v>
+        <v>12.57805347442627</v>
       </c>
       <c r="Z2" t="n">
-        <v>1.035713911056519</v>
+        <v>1.071682453155518</v>
       </c>
       <c r="AA2" t="n">
-        <v>4.443002700805664</v>
+        <v>14.45655345916748</v>
       </c>
       <c r="AB2" t="n">
-        <v>3.948645353317261</v>
+        <v>1.242449760437012</v>
       </c>
       <c r="AC2" t="n">
-        <v>-11.86921405792236</v>
+        <v>-11.70841598510742</v>
       </c>
       <c r="AD2" t="n">
-        <v>-2.026759147644043</v>
+        <v>-1.86942446231842</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.01705215126276016</v>
+        <v>0.05076132342219353</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.39617395401001</v>
+        <v>2.604483604431152</v>
       </c>
       <c r="AG2" t="n">
-        <v>1.247585415840149</v>
+        <v>1.302456736564636</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.8548141717910767</v>
+        <v>0.939742386341095</v>
       </c>
       <c r="AI2" t="n">
-        <v>7.240087985992432</v>
+        <v>6.340747356414795</v>
       </c>
       <c r="AJ2" t="n">
-        <v>1.097067594528198</v>
+        <v>0.7994276285171509</v>
       </c>
       <c r="AK2" t="n">
-        <v>21.1597728729248</v>
+        <v>7.211807727813721</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.263010025024414</v>
+        <v>1.52609121799469</v>
       </c>
       <c r="AM2" t="n">
-        <v>29.3732852935791</v>
+        <v>27.38559722900391</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.3709474802017212</v>
+        <v>0.414627879858017</v>
       </c>
       <c r="AO2" t="n">
-        <v>511.8189697265625</v>
+        <v>521.3392944335938</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.3724395930767059</v>
+        <v>0.4843678176403046</v>
       </c>
       <c r="AQ2" t="n">
-        <v>1203.272583007812</v>
+        <v>1103.441772460938</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.2456410080194473</v>
+        <v>0.2263720780611038</v>
       </c>
       <c r="AS2" t="n">
-        <v>-53.89140319824219</v>
+        <v>-64.62120819091797</v>
       </c>
       <c r="AT2" t="n">
-        <v>-1.429143786430359</v>
+        <v>-1.349149227142334</v>
       </c>
       <c r="AU2" t="n">
-        <v>1524.739624023438</v>
+        <v>1526.146240234375</v>
       </c>
       <c r="AV2" t="n">
-        <v>0.2074335515499115</v>
+        <v>0.2344062328338623</v>
       </c>
       <c r="AW2" t="n">
-        <v>857.173095703125</v>
+        <v>854.1484985351562</v>
       </c>
       <c r="AX2" t="n">
-        <v>0.3642056584358215</v>
+        <v>0.4293943643569946</v>
       </c>
       <c r="AY2" t="n">
-        <v>-50.71536254882812</v>
+        <v>-74.64289855957031</v>
       </c>
       <c r="AZ2" t="n">
-        <v>-1.18555223941803</v>
+        <v>-1.029463410377502</v>
       </c>
       <c r="BA2" t="n">
-        <v>2792.530029296875</v>
+        <v>2656.90673828125</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.1327045857906342</v>
+        <v>0.1229096576571465</v>
       </c>
       <c r="BC2" t="n">
-        <v>574.93408203125</v>
+        <v>555.29345703125</v>
       </c>
       <c r="BD2" t="n">
-        <v>0.623511016368866</v>
+        <v>0.6560559868812561</v>
       </c>
       <c r="BE2" t="n">
-        <v>-56.62160110473633</v>
+        <v>-77.67434692382812</v>
       </c>
       <c r="BF2" t="n">
-        <v>-1.014002323150635</v>
+        <v>-0.9611384272575378</v>
       </c>
       <c r="BG2" t="n">
-        <v>-18.72908973693848</v>
+        <v>-17.49964714050293</v>
       </c>
       <c r="BH2" t="n">
-        <v>-0.4859675467014313</v>
+        <v>-0.59625244140625</v>
       </c>
       <c r="BI2" t="n">
-        <v>29.47310447692871</v>
+        <v>25.24982643127441</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.3379878997802734</v>
+        <v>0.4785923957824707</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.09464066475629807</v>
+        <v>0.08542526513338089</v>
       </c>
       <c r="BL2" t="n">
-        <v>0.2965871095657349</v>
+        <v>0.3522613048553467</v>
       </c>
       <c r="BM2" t="n">
-        <v>-0.02190934307873249</v>
+        <v>-0.02931478805840015</v>
       </c>
       <c r="BN2" t="n">
-        <v>-0.5793618559837341</v>
+        <v>-0.4766077101230621</v>
       </c>
       <c r="BO2" t="n">
-        <v>1.101303458213806</v>
+        <v>0.7294573783874512</v>
       </c>
       <c r="BP2" t="n">
-        <v>0.7838082909584045</v>
+        <v>0.8740352988243103</v>
       </c>
       <c r="BQ2" t="n">
-        <v>29.50015830993652</v>
+        <v>30.09926986694336</v>
       </c>
       <c r="BR2" t="n">
-        <v>0.5549203157424927</v>
+        <v>0.5807392001152039</v>
       </c>
       <c r="BS2" t="n">
-        <v>14.05053329467773</v>
+        <v>11.88765430450439</v>
       </c>
       <c r="BT2" t="n">
-        <v>0.9970332980155945</v>
+        <v>1.088986754417419</v>
       </c>
       <c r="BU2" t="n">
-        <v>5.558104038238525</v>
+        <v>16.62846565246582</v>
       </c>
       <c r="BV2" t="n">
-        <v>3.337806940078735</v>
+        <v>1.074229121208191</v>
       </c>
       <c r="BW2" t="n">
-        <v>-16.89686012268066</v>
+        <v>-19.99944305419922</v>
       </c>
       <c r="BX2" t="n">
-        <v>-1.345267057418823</v>
+        <v>-0.9780746102333069</v>
       </c>
       <c r="BY2" t="n">
-        <v>-8.762996673583984</v>
+        <v>-3.50093150138855</v>
       </c>
       <c r="BZ2" t="n">
-        <v>18.4128303527832</v>
+        <v>10.26154899597168</v>
       </c>
       <c r="CA2" t="n">
-        <v>0.09589102119207382</v>
+        <v>0.0543997548520565</v>
       </c>
       <c r="CB2" t="n">
-        <v>-0.006538162473589182</v>
+        <v>-0.004938334226608276</v>
       </c>
       <c r="CC2" t="n">
-        <v>0.1371414214372635</v>
+        <v>0.1325622051954269</v>
       </c>
       <c r="CD2" t="n">
-        <v>3.964757680892944</v>
+        <v>4.329896926879883</v>
       </c>
       <c r="CE2" t="n">
-        <v>3.15315318107605</v>
+        <v>2.296450853347778</v>
       </c>
       <c r="CF2" t="n">
-        <v>0.2557142674922943</v>
+        <v>0.2972727119922638</v>
       </c>
       <c r="CG2" t="n">
-        <v>0.2637562155723572</v>
+        <v>0.2350276708602905</v>
       </c>
       <c r="CH2" t="n">
-        <v>0.04833333566784859</v>
+        <v>0.09692307561635971</v>
       </c>
       <c r="CI2" t="n">
-        <v>0.01462494023144245</v>
+        <v>0.09626761823892593</v>
       </c>
       <c r="CJ2" t="n">
-        <v>-16.60617828369141</v>
+        <v>-25.15578269958496</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated fetch API endpoint
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -872,268 +872,268 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>32.37878799438477</v>
+        <v>37.14665222167969</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1399308443069458</v>
+        <v>0.08998681604862213</v>
       </c>
       <c r="C2" t="n">
-        <v>31.48935699462891</v>
+        <v>36.28823852539062</v>
       </c>
       <c r="D2" t="n">
-        <v>32.65531539916992</v>
+        <v>38.21646499633789</v>
       </c>
       <c r="E2" t="n">
-        <v>33.95757675170898</v>
+        <v>39.44939422607422</v>
       </c>
       <c r="F2" t="n">
-        <v>2.468219757080078</v>
+        <v>3.161155700683594</v>
       </c>
       <c r="G2" t="n">
-        <v>123.0326080322266</v>
+        <v>117.2871627807617</v>
       </c>
       <c r="H2" t="n">
-        <v>97.15403747558594</v>
+        <v>92.78736877441406</v>
       </c>
       <c r="I2" t="n">
-        <v>26.1563606262207</v>
+        <v>9.692314147949219</v>
       </c>
       <c r="J2" t="n">
-        <v>14.35910224914551</v>
+        <v>5.844415664672852</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7915711402893066</v>
+        <v>1.161906838417053</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7487615942955017</v>
+        <v>0.7524440288543701</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2599876224994659</v>
+        <v>0.3623009920120239</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6808357238769531</v>
+        <v>1.033462285995483</v>
       </c>
       <c r="O2" t="n">
-        <v>1.196025133132935</v>
+        <v>1.761012315750122</v>
       </c>
       <c r="P2" t="n">
-        <v>0.936037540435791</v>
+        <v>1.398711323738098</v>
       </c>
       <c r="Q2" t="n">
-        <v>16.84541511535645</v>
+        <v>11.63771629333496</v>
       </c>
       <c r="R2" t="n">
-        <v>12.32826614379883</v>
+        <v>5.699487209320068</v>
       </c>
       <c r="S2" t="n">
-        <v>10.85582828521729</v>
+        <v>11.84694671630859</v>
       </c>
       <c r="T2" t="n">
-        <v>8.22602653503418</v>
+        <v>5.24303674697876</v>
       </c>
       <c r="U2" t="n">
-        <v>0.5492869019508362</v>
+        <v>0.7891900539398193</v>
       </c>
       <c r="V2" t="n">
-        <v>1.099833011627197</v>
+        <v>1.155808091163635</v>
       </c>
       <c r="W2" t="n">
-        <v>21.01264381408691</v>
+        <v>27.03838920593262</v>
       </c>
       <c r="X2" t="n">
-        <v>1.111422657966614</v>
+        <v>0.7595821022987366</v>
       </c>
       <c r="Y2" t="n">
-        <v>12.57805347442627</v>
+        <v>8.101020812988281</v>
       </c>
       <c r="Z2" t="n">
-        <v>1.071682453155518</v>
+        <v>1.850481271743774</v>
       </c>
       <c r="AA2" t="n">
-        <v>14.45655345916748</v>
+        <v>-3.723021507263184</v>
       </c>
       <c r="AB2" t="n">
-        <v>1.242449760437012</v>
+        <v>-5.016207218170166</v>
       </c>
       <c r="AC2" t="n">
-        <v>-11.70841598510742</v>
+        <v>-25.08605766296387</v>
       </c>
       <c r="AD2" t="n">
-        <v>-1.86942446231842</v>
+        <v>-0.9569094777107239</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.05076132342219353</v>
+        <v>0.01194771099835634</v>
       </c>
       <c r="AF2" t="n">
-        <v>2.604483604431152</v>
+        <v>1.887701511383057</v>
       </c>
       <c r="AG2" t="n">
-        <v>1.302456736564636</v>
+        <v>0.8703248500823975</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.939742386341095</v>
+        <v>0.955550491809845</v>
       </c>
       <c r="AI2" t="n">
-        <v>6.340747356414795</v>
+        <v>10.58922576904297</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.7994276285171509</v>
+        <v>0.503117561340332</v>
       </c>
       <c r="AK2" t="n">
-        <v>7.211807727813721</v>
+        <v>12.16113376617432</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.52609121799469</v>
+        <v>1.477150440216064</v>
       </c>
       <c r="AM2" t="n">
-        <v>27.38559722900391</v>
+        <v>30.17942047119141</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.414627879858017</v>
+        <v>0.5507754683494568</v>
       </c>
       <c r="AO2" t="n">
-        <v>521.3392944335938</v>
+        <v>504.2869262695312</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.4843678176403046</v>
+        <v>0.3689597547054291</v>
       </c>
       <c r="AQ2" t="n">
-        <v>1103.441772460938</v>
+        <v>1263.915161132812</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.2263720780611038</v>
+        <v>0.1885583698749542</v>
       </c>
       <c r="AS2" t="n">
-        <v>-64.62120819091797</v>
+        <v>-61.3365592956543</v>
       </c>
       <c r="AT2" t="n">
-        <v>-1.349149227142334</v>
+        <v>-1.426013350486755</v>
       </c>
       <c r="AU2" t="n">
-        <v>1526.146240234375</v>
+        <v>1443.920776367188</v>
       </c>
       <c r="AV2" t="n">
-        <v>0.2344062328338623</v>
+        <v>0.2011489421129227</v>
       </c>
       <c r="AW2" t="n">
-        <v>854.1484985351562</v>
+        <v>926.939697265625</v>
       </c>
       <c r="AX2" t="n">
-        <v>0.4293943643569946</v>
+        <v>0.3854619562625885</v>
       </c>
       <c r="AY2" t="n">
-        <v>-74.64289855957031</v>
+        <v>-52.97447204589844</v>
       </c>
       <c r="AZ2" t="n">
-        <v>-1.029463410377502</v>
+        <v>-1.290053009986877</v>
       </c>
       <c r="BA2" t="n">
-        <v>2656.90673828125</v>
+        <v>2631.161865234375</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.1229096576571465</v>
+        <v>0.1230771988630295</v>
       </c>
       <c r="BC2" t="n">
-        <v>555.29345703125</v>
+        <v>557.8199462890625</v>
       </c>
       <c r="BD2" t="n">
-        <v>0.6560559868812561</v>
+        <v>0.5859470963478088</v>
       </c>
       <c r="BE2" t="n">
-        <v>-77.67434692382812</v>
+        <v>-59.26141357421875</v>
       </c>
       <c r="BF2" t="n">
-        <v>-0.9611384272575378</v>
+        <v>-1.092938542366028</v>
       </c>
       <c r="BG2" t="n">
-        <v>-17.49964714050293</v>
+        <v>-18.54858016967773</v>
       </c>
       <c r="BH2" t="n">
-        <v>-0.59625244140625</v>
+        <v>-0.4067893922328949</v>
       </c>
       <c r="BI2" t="n">
-        <v>25.24982643127441</v>
+        <v>29.83827018737793</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.4785923957824707</v>
+        <v>0.3367993235588074</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.08542526513338089</v>
+        <v>0.1054705381393433</v>
       </c>
       <c r="BL2" t="n">
-        <v>0.3522613048553467</v>
+        <v>0.3011460602283478</v>
       </c>
       <c r="BM2" t="n">
-        <v>-0.02931478805840015</v>
+        <v>-0.03149436786770821</v>
       </c>
       <c r="BN2" t="n">
-        <v>-0.4766077101230621</v>
+        <v>-0.3907376825809479</v>
       </c>
       <c r="BO2" t="n">
-        <v>0.7294573783874512</v>
+        <v>0.9747639894485474</v>
       </c>
       <c r="BP2" t="n">
-        <v>0.8740352988243103</v>
+        <v>0.9649931788444519</v>
       </c>
       <c r="BQ2" t="n">
-        <v>30.09926986694336</v>
+        <v>34.11368560791016</v>
       </c>
       <c r="BR2" t="n">
-        <v>0.5807392001152039</v>
+        <v>0.3914794325828552</v>
       </c>
       <c r="BS2" t="n">
-        <v>11.88765430450439</v>
+        <v>5.269437313079834</v>
       </c>
       <c r="BT2" t="n">
-        <v>1.088986754417419</v>
+        <v>2.6060950756073</v>
       </c>
       <c r="BU2" t="n">
-        <v>16.62846565246582</v>
+        <v>-3.29999852180481</v>
       </c>
       <c r="BV2" t="n">
-        <v>1.074229121208191</v>
+        <v>-5.763919353485107</v>
       </c>
       <c r="BW2" t="n">
-        <v>-19.99944305419922</v>
+        <v>-33.51142501831055</v>
       </c>
       <c r="BX2" t="n">
-        <v>-0.9780746102333069</v>
+        <v>-0.5464003086090088</v>
       </c>
       <c r="BY2" t="n">
-        <v>-3.50093150138855</v>
+        <v>-5.634957313537598</v>
       </c>
       <c r="BZ2" t="n">
-        <v>10.26154899597168</v>
+        <v>10.7114429473877</v>
       </c>
       <c r="CA2" t="n">
-        <v>0.0543997548520565</v>
+        <v>0.05253883451223373</v>
       </c>
       <c r="CB2" t="n">
-        <v>-0.004938334226608276</v>
+        <v>-0.006608311552554369</v>
       </c>
       <c r="CC2" t="n">
-        <v>0.1325622051954269</v>
+        <v>0.08324876427650452</v>
       </c>
       <c r="CD2" t="n">
-        <v>4.329896926879883</v>
+        <v>3.344481706619263</v>
       </c>
       <c r="CE2" t="n">
-        <v>2.296450853347778</v>
+        <v>1.700680375099182</v>
       </c>
       <c r="CF2" t="n">
-        <v>0.2972727119922638</v>
+        <v>0.465999960899353</v>
       </c>
       <c r="CG2" t="n">
-        <v>0.2350276708602905</v>
+        <v>0.2447529286146164</v>
       </c>
       <c r="CH2" t="n">
-        <v>0.09692307561635971</v>
+        <v>0.08166667073965073</v>
       </c>
       <c r="CI2" t="n">
-        <v>0.09626761823892593</v>
+        <v>0.06792560964822769</v>
       </c>
       <c r="CJ2" t="n">
-        <v>-25.15578269958496</v>
+        <v>-17.85830497741699</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move app.py to backend folder
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -872,268 +872,268 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>37.14665222167969</v>
+        <v>18.71833038330078</v>
       </c>
       <c r="B2" t="n">
-        <v>0.08998681604862213</v>
+        <v>0.4376151561737061</v>
       </c>
       <c r="C2" t="n">
-        <v>36.28823852539062</v>
+        <v>13.29975414276123</v>
       </c>
       <c r="D2" t="n">
-        <v>38.21646499633789</v>
+        <v>13.82852172851562</v>
       </c>
       <c r="E2" t="n">
-        <v>39.44939422607422</v>
+        <v>25.80756568908691</v>
       </c>
       <c r="F2" t="n">
-        <v>3.161155700683594</v>
+        <v>12.50781154632568</v>
       </c>
       <c r="G2" t="n">
-        <v>117.2871627807617</v>
+        <v>21.36471557617188</v>
       </c>
       <c r="H2" t="n">
-        <v>92.78736877441406</v>
+        <v>18.25589752197266</v>
       </c>
       <c r="I2" t="n">
-        <v>9.692314147949219</v>
+        <v>96.32051086425781</v>
       </c>
       <c r="J2" t="n">
-        <v>5.844415664672852</v>
+        <v>17.66203689575195</v>
       </c>
       <c r="K2" t="n">
-        <v>1.161906838417053</v>
+        <v>0.7296184301376343</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7524440288543701</v>
+        <v>0.5878180861473083</v>
       </c>
       <c r="M2" t="n">
-        <v>0.3623009920120239</v>
+        <v>0.4399476051330566</v>
       </c>
       <c r="N2" t="n">
-        <v>1.033462285995483</v>
+        <v>0.5548169612884521</v>
       </c>
       <c r="O2" t="n">
-        <v>1.761012315750122</v>
+        <v>1.096246123313904</v>
       </c>
       <c r="P2" t="n">
-        <v>1.398711323738098</v>
+        <v>0.6562985181808472</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.63771629333496</v>
+        <v>6.152434825897217</v>
       </c>
       <c r="R2" t="n">
-        <v>5.699487209320068</v>
+        <v>4.03209400177002</v>
       </c>
       <c r="S2" t="n">
-        <v>11.84694671630859</v>
+        <v>7.453845500946045</v>
       </c>
       <c r="T2" t="n">
-        <v>5.24303674697876</v>
+        <v>4.290507793426514</v>
       </c>
       <c r="U2" t="n">
-        <v>0.7891900539398193</v>
+        <v>0.7141743302345276</v>
       </c>
       <c r="V2" t="n">
-        <v>1.155808091163635</v>
+        <v>0.6739721298217773</v>
       </c>
       <c r="W2" t="n">
-        <v>27.03838920593262</v>
+        <v>26.18112373352051</v>
       </c>
       <c r="X2" t="n">
-        <v>0.7595821022987366</v>
+        <v>0.4668290913105011</v>
       </c>
       <c r="Y2" t="n">
-        <v>8.101020812988281</v>
+        <v>17.55410957336426</v>
       </c>
       <c r="Z2" t="n">
-        <v>1.850481271743774</v>
+        <v>0.5447753667831421</v>
       </c>
       <c r="AA2" t="n">
-        <v>-3.723021507263184</v>
+        <v>-2.129408121109009</v>
       </c>
       <c r="AB2" t="n">
-        <v>-5.016207218170166</v>
+        <v>-4.836315631866455</v>
       </c>
       <c r="AC2" t="n">
-        <v>-25.08605766296387</v>
+        <v>-0.7592475414276123</v>
       </c>
       <c r="AD2" t="n">
-        <v>-0.9569094777107239</v>
+        <v>-28.99734687805176</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.01194771099835634</v>
+        <v>0.1064426675438881</v>
       </c>
       <c r="AF2" t="n">
-        <v>1.887701511383057</v>
+        <v>1.857770085334778</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.8703248500823975</v>
+        <v>1.802153587341309</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.955550491809845</v>
+        <v>0.5884233713150024</v>
       </c>
       <c r="AI2" t="n">
-        <v>10.58922576904297</v>
+        <v>-1.168940782546997</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.503117561340332</v>
+        <v>-3.568675994873047</v>
       </c>
       <c r="AK2" t="n">
-        <v>12.16113376617432</v>
+        <v>7.673895359039307</v>
       </c>
       <c r="AL2" t="n">
-        <v>1.477150440216064</v>
+        <v>2.939530372619629</v>
       </c>
       <c r="AM2" t="n">
-        <v>30.17942047119141</v>
+        <v>27.7790584564209</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.5507754683494568</v>
+        <v>0.4332564473152161</v>
       </c>
       <c r="AO2" t="n">
-        <v>504.2869262695312</v>
+        <v>720.9705200195312</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.3689597547054291</v>
+        <v>0.2956345677375793</v>
       </c>
       <c r="AQ2" t="n">
-        <v>1263.915161132812</v>
+        <v>1247.053100585938</v>
       </c>
       <c r="AR2" t="n">
-        <v>0.1885583698749542</v>
+        <v>0.192892923951149</v>
       </c>
       <c r="AS2" t="n">
-        <v>-61.3365592956543</v>
+        <v>-12.87798500061035</v>
       </c>
       <c r="AT2" t="n">
-        <v>-1.426013350486755</v>
+        <v>-1.991369843482971</v>
       </c>
       <c r="AU2" t="n">
-        <v>1443.920776367188</v>
+        <v>1751.251586914062</v>
       </c>
       <c r="AV2" t="n">
-        <v>0.2011489421129227</v>
+        <v>0.1893404424190521</v>
       </c>
       <c r="AW2" t="n">
-        <v>926.939697265625</v>
+        <v>960.4345703125</v>
       </c>
       <c r="AX2" t="n">
-        <v>0.3854619562625885</v>
+        <v>0.344479501247406</v>
       </c>
       <c r="AY2" t="n">
-        <v>-52.97447204589844</v>
+        <v>-22.43215179443359</v>
       </c>
       <c r="AZ2" t="n">
-        <v>-1.290053009986877</v>
+        <v>-0.9704205989837646</v>
       </c>
       <c r="BA2" t="n">
-        <v>2631.161865234375</v>
+        <v>2967.92333984375</v>
       </c>
       <c r="BB2" t="n">
-        <v>0.1230771988630295</v>
+        <v>0.1067371517419815</v>
       </c>
       <c r="BC2" t="n">
-        <v>557.8199462890625</v>
+        <v>743.931884765625</v>
       </c>
       <c r="BD2" t="n">
-        <v>0.5859470963478088</v>
+        <v>0.6883451342582703</v>
       </c>
       <c r="BE2" t="n">
-        <v>-59.26141357421875</v>
+        <v>-29.1151237487793</v>
       </c>
       <c r="BF2" t="n">
-        <v>-1.092938542366028</v>
+        <v>-0.7102044820785522</v>
       </c>
       <c r="BG2" t="n">
-        <v>-18.54858016967773</v>
+        <v>-17.00508499145508</v>
       </c>
       <c r="BH2" t="n">
-        <v>-0.4067893922328949</v>
+        <v>-0.3740938305854797</v>
       </c>
       <c r="BI2" t="n">
-        <v>29.83827018737793</v>
+        <v>29.55185699462891</v>
       </c>
       <c r="BJ2" t="n">
-        <v>0.3367993235588074</v>
+        <v>0.3286204934120178</v>
       </c>
       <c r="BK2" t="n">
-        <v>0.1054705381393433</v>
+        <v>-0.02282265201210976</v>
       </c>
       <c r="BL2" t="n">
-        <v>0.3011460602283478</v>
+        <v>-2.408941507339478</v>
       </c>
       <c r="BM2" t="n">
-        <v>-0.03149436786770821</v>
+        <v>-0.01756853424012661</v>
       </c>
       <c r="BN2" t="n">
-        <v>-0.3907376825809479</v>
+        <v>-1.024107336997986</v>
       </c>
       <c r="BO2" t="n">
-        <v>0.9747639894485474</v>
+        <v>0.6996985077857971</v>
       </c>
       <c r="BP2" t="n">
-        <v>0.9649931788444519</v>
+        <v>0.7056123018264771</v>
       </c>
       <c r="BQ2" t="n">
-        <v>34.11368560791016</v>
+        <v>25.67791748046875</v>
       </c>
       <c r="BR2" t="n">
-        <v>0.3914794325828552</v>
+        <v>0.4899005889892578</v>
       </c>
       <c r="BS2" t="n">
-        <v>5.269437313079834</v>
+        <v>18.38669776916504</v>
       </c>
       <c r="BT2" t="n">
-        <v>2.6060950756073</v>
+        <v>0.50506192445755</v>
       </c>
       <c r="BU2" t="n">
-        <v>-3.29999852180481</v>
+        <v>-2.624396800994873</v>
       </c>
       <c r="BV2" t="n">
-        <v>-5.763919353485107</v>
+        <v>-3.945217847824097</v>
       </c>
       <c r="BW2" t="n">
-        <v>-33.51142501831055</v>
+        <v>-0.9146479368209839</v>
       </c>
       <c r="BX2" t="n">
-        <v>-0.5464003086090088</v>
+        <v>-24.84650802612305</v>
       </c>
       <c r="BY2" t="n">
-        <v>-5.634957313537598</v>
+        <v>-21.01335334777832</v>
       </c>
       <c r="BZ2" t="n">
-        <v>10.7114429473877</v>
+        <v>31.87785911560059</v>
       </c>
       <c r="CA2" t="n">
-        <v>0.05253883451223373</v>
+        <v>0.01009888760745525</v>
       </c>
       <c r="CB2" t="n">
-        <v>-0.006608311552554369</v>
+        <v>-0.01251515280455351</v>
       </c>
       <c r="CC2" t="n">
-        <v>0.08324876427650452</v>
+        <v>0.7081084251403809</v>
       </c>
       <c r="CD2" t="n">
-        <v>3.344481706619263</v>
+        <v>2.521008491516113</v>
       </c>
       <c r="CE2" t="n">
-        <v>1.700680375099182</v>
+        <v>0.8849557638168335</v>
       </c>
       <c r="CF2" t="n">
-        <v>0.465999960899353</v>
+        <v>1.079999923706055</v>
       </c>
       <c r="CG2" t="n">
-        <v>0.2447529286146164</v>
+        <v>0</v>
       </c>
       <c r="CH2" t="n">
-        <v>0.08166667073965073</v>
+        <v>0</v>
       </c>
       <c r="CI2" t="n">
-        <v>0.06792560964822769</v>
+        <v>0</v>
       </c>
       <c r="CJ2" t="n">
-        <v>-17.85830497741699</v>
+        <v>-25.62125968933105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>